<commit_message>
converted xlxs files to csv
</commit_message>
<xml_diff>
--- a/Paper_retrieval.xlsx
+++ b/Paper_retrieval.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniluxembourg-my.sharepoint.com/personal/laura_bernardy_uni_lu/Documents/Documents/GitHub/DarkJargon-SOK-USENIX26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{8F195C7A-5350-41BC-8581-EC68EBF45E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23020854-605B-4ADB-B74C-D7AE8FEBC51F}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{8F195C7A-5350-41BC-8581-EC68EBF45E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47F17C1F-905E-43A8-827B-65ABE7987E55}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{EA17AA5D-E7D2-4D66-90DD-3C232CE04C93}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA17AA5D-E7D2-4D66-90DD-3C232CE04C93}"/>
   </bookViews>
   <sheets>
     <sheet name="search_full_results" sheetId="3" r:id="rId1"/>
@@ -18,15 +18,28 @@
     <sheet name="snowballing_dedup_results" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">search_dedup_results!$O$1:$O$848</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">search_dedup_results!$A$1:$P$848</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">snowballing_dedup_results!$O$1:$O$42</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13545" uniqueCount="4750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13546" uniqueCount="4751">
   <si>
     <t>Item Type</t>
   </si>
@@ -14276,13 +14289,16 @@
   </si>
   <si>
     <t>https://www.dea.gov/documents/2018/2018-07/2018-07-01/2018-slang-terms-and-code-words</t>
+  </si>
+  <si>
+    <t>Usenix</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -14413,6 +14429,20 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -14715,7 +14745,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -14758,8 +14788,9 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment shrinkToFit="1"/>
@@ -14768,50 +14799,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+  <cellStyles count="43">
+    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Akzent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Akzent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Akzent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Akzent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Akzent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Akzent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Ausgabe" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Berechnung" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Eingabe" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Link" xfId="42" builtinId="8"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Überschrift 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Warnender Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -14831,7 +14865,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -15148,7 +15182,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A26FC26A-A1E7-4AFF-9612-456554910556}">
   <dimension ref="A1:CG866"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="69.6640625" customWidth="1"/>
   </cols>
@@ -49461,12 +49495,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BE0D9D0-4103-4D14-9E1F-AE6ADFAADF9D}">
   <dimension ref="A1:P848"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="111" customWidth="1"/>
-    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="4" max="4" width="72.44140625" customWidth="1"/>
+    <col min="5" max="5" width="45.21875" customWidth="1"/>
     <col min="6" max="6" width="2.88671875" customWidth="1"/>
-    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="7" max="7" width="6.44140625" customWidth="1"/>
+    <col min="9" max="9" width="34.5546875" customWidth="1"/>
     <col min="10" max="10" width="8.88671875" style="1"/>
     <col min="11" max="11" width="3.6640625" customWidth="1"/>
     <col min="12" max="12" width="54.21875" customWidth="1"/>
@@ -49591,7 +49626,7 @@
       <c r="H3" t="s">
         <v>29</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="6" t="s">
         <v>30</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -68282,8 +68317,8 @@
       <c r="N648" s="1" t="s">
         <v>2356</v>
       </c>
-      <c r="O648" t="s">
-        <v>3317</v>
+      <c r="P648" t="s">
+        <v>3322</v>
       </c>
     </row>
     <row r="649" spans="1:16" x14ac:dyDescent="0.3">
@@ -74102,19 +74137,26 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="O1:O848" xr:uid="{7BE0D9D0-4103-4D14-9E1F-AE6ADFAADF9D}"/>
+  <hyperlinks>
+    <hyperlink ref="I3" r:id="rId1" xr:uid="{35FFA5EC-1206-4DCD-8D27-6E81D93B4D02}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6838546E-B76C-4CCB-8F31-DD3110A994D5}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:P42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="64.6640625" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" customWidth="1"/>
+    <col min="4" max="4" width="86.109375" customWidth="1"/>
+    <col min="6" max="6" width="6.21875" customWidth="1"/>
+    <col min="7" max="7" width="0.5546875" customWidth="1"/>
+    <col min="8" max="8" width="4.33203125" customWidth="1"/>
+    <col min="9" max="9" width="72.77734375" customWidth="1"/>
+    <col min="10" max="10" width="30.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
@@ -74167,7 +74209,7 @@
         <v>3319</v>
       </c>
     </row>
-    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -74205,7 +74247,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -74243,7 +74285,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -74281,7 +74323,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -74319,7 +74361,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -74354,7 +74396,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -74386,7 +74428,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -74434,6 +74476,9 @@
       <c r="D9" t="s">
         <v>3339</v>
       </c>
+      <c r="E9" t="s">
+        <v>4750</v>
+      </c>
       <c r="I9" t="s">
         <v>3340</v>
       </c>
@@ -74457,7 +74502,7 @@
       <c r="C10" t="s">
         <v>3342</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="7" t="s">
         <v>3343</v>
       </c>
       <c r="E10" t="s">
@@ -74482,7 +74527,7 @@
         <v>3317</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -74514,7 +74559,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -74549,7 +74594,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -74575,7 +74620,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -74610,7 +74655,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -74645,7 +74690,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>43</v>
       </c>
@@ -74680,7 +74725,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -74715,7 +74760,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -74747,7 +74792,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -74779,7 +74824,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -74814,7 +74859,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -74849,7 +74894,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -74884,7 +74929,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -74922,7 +74967,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -74967,10 +75012,10 @@
       <c r="C25" t="s">
         <v>3437</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="7" t="s">
         <v>3438</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="6" t="s">
         <v>3439</v>
       </c>
       <c r="J25" t="s">
@@ -74983,7 +75028,7 @@
         <v>3317</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -74993,7 +75038,7 @@
       <c r="C26" t="s">
         <v>3441</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="7" t="s">
         <v>3442</v>
       </c>
       <c r="E26" t="s">
@@ -75018,7 +75063,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -75028,7 +75073,7 @@
       <c r="C27" t="s">
         <v>3447</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="7" t="s">
         <v>3448</v>
       </c>
       <c r="E27" t="s">
@@ -75053,7 +75098,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -75063,7 +75108,7 @@
       <c r="C28" t="s">
         <v>3454</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="7" t="s">
         <v>3455</v>
       </c>
       <c r="E28" t="s">
@@ -75088,7 +75133,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -75098,7 +75143,7 @@
       <c r="C29" t="s">
         <v>3460</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="7" t="s">
         <v>3461</v>
       </c>
       <c r="E29" t="s">
@@ -75123,7 +75168,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -75133,7 +75178,7 @@
       <c r="C30" t="s">
         <v>3467</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="7" t="s">
         <v>3468</v>
       </c>
       <c r="E30" t="s">
@@ -75168,7 +75213,7 @@
       <c r="C31" t="s">
         <v>3472</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="7" t="s">
         <v>3473</v>
       </c>
       <c r="H31" t="s">
@@ -75190,7 +75235,7 @@
         <v>3317</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -75200,7 +75245,7 @@
       <c r="C32" t="s">
         <v>3477</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="7" t="s">
         <v>3478</v>
       </c>
       <c r="E32" t="s">
@@ -75225,7 +75270,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -75235,7 +75280,7 @@
       <c r="C33" t="s">
         <v>3483</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="7" t="s">
         <v>3484</v>
       </c>
       <c r="E33" t="s">
@@ -75273,7 +75318,7 @@
       <c r="C34" t="s">
         <v>2437</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="7" t="s">
         <v>3488</v>
       </c>
       <c r="E34" t="s">
@@ -75298,7 +75343,7 @@
         <v>3317</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -75308,7 +75353,7 @@
       <c r="C35" t="s">
         <v>3494</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="7" t="s">
         <v>3495</v>
       </c>
       <c r="E35" t="s">
@@ -75333,7 +75378,7 @@
         <v>3322</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -75343,7 +75388,7 @@
       <c r="C36" t="s">
         <v>3500</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="7" t="s">
         <v>3501</v>
       </c>
       <c r="E36" t="s">
@@ -75378,7 +75423,7 @@
       <c r="C37" t="s">
         <v>3506</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="7" t="s">
         <v>3507</v>
       </c>
       <c r="E37" t="s">
@@ -75406,7 +75451,7 @@
         <v>3325</v>
       </c>
     </row>
-    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -75416,7 +75461,7 @@
       <c r="C38" t="s">
         <v>3511</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="7" t="s">
         <v>3512</v>
       </c>
       <c r="E38" t="s">
@@ -75451,7 +75496,7 @@
       <c r="C39" t="s">
         <v>3518</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="7" t="s">
         <v>3519</v>
       </c>
       <c r="E39" t="s">
@@ -75476,7 +75521,7 @@
         <v>3317</v>
       </c>
     </row>
-    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -75486,7 +75531,7 @@
       <c r="C40" t="s">
         <v>3525</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="7" t="s">
         <v>3526</v>
       </c>
       <c r="E40" t="s">
@@ -75515,7 +75560,7 @@
       <c r="A41" t="s">
         <v>4745</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="7" t="s">
         <v>4746</v>
       </c>
       <c r="I41" t="s">
@@ -75529,7 +75574,7 @@
       <c r="A42" t="s">
         <v>4745</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="7" t="s">
         <v>4747</v>
       </c>
       <c r="I42" t="s">
@@ -75539,14 +75584,13 @@
         <v>3317</v>
       </c>
     </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="D43" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="O1:O42" xr:uid="{6838546E-B76C-4CCB-8F31-DD3110A994D5}">
-    <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="I25" r:id="rId1" xr:uid="{7EB0222D-CB80-4457-A0A8-047C41516DD5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>